<commit_message>
data: rebuild analysis on Stack Overflow Developer Survey 2025 (49,191 respondents)
- analysis/recompute_from_survey.py: recompute tables from latest survey, same logic
- analysis/market_data.json: computed signals (language/database/salary/role/country)
- market_insight_data.py now loads live numbers; regenerate dashboard/pptx/sql/pbip/CSVs
- IDE kept from last survey that asked it (2025 dropped the IDE question)
</commit_message>
<xml_diff>
--- a/data/clean/skill_market_insight.xlsx
+++ b/data/clean/skill_market_insight.xlsx
@@ -451,7 +451,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>11552</v>
+        <v>49191</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -466,7 +466,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>135</v>
+        <v>177</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>12</v>
+        <v>145</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -496,7 +496,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>57844</v>
+        <v>75320</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>96.2</v>
+        <v>0</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -537,11 +537,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Avg languages worked per respondent</t>
+          <t>Average languages worked per respondent</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5.2</v>
+        <v>4</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -552,11 +552,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Avg languages desired per respondent</t>
+          <t>Average languages desired per respondent</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4.9</v>
+        <v>2.8</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -902,7 +902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -945,23 +945,23 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>JavaScript</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>8805</v>
+        <v>18410</v>
       </c>
       <c r="C2" t="n">
-        <v>6715</v>
+        <v>12419</v>
       </c>
       <c r="D2" t="n">
-        <v>-2090</v>
+        <v>-5991</v>
       </c>
       <c r="E2" t="n">
-        <v>-23.7</v>
+        <v>-32.5</v>
       </c>
       <c r="F2" t="n">
-        <v>58.1</v>
+        <v>25.2</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -972,23 +972,23 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HTML/CSS</t>
+          <t>SQL</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7920</v>
+        <v>18633</v>
       </c>
       <c r="C3" t="n">
-        <v>5398</v>
+        <v>11257</v>
       </c>
       <c r="D3" t="n">
-        <v>-2522</v>
+        <v>-7376</v>
       </c>
       <c r="E3" t="n">
-        <v>-31.8</v>
+        <v>-39.6</v>
       </c>
       <c r="F3" t="n">
-        <v>46.7</v>
+        <v>22.9</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -999,50 +999,50 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>HTML/CSS</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4611</v>
+        <v>19698</v>
       </c>
       <c r="C4" t="n">
-        <v>5309</v>
+        <v>10661</v>
       </c>
       <c r="D4" t="n">
-        <v>698</v>
+        <v>-9037</v>
       </c>
       <c r="E4" t="n">
-        <v>15.1</v>
+        <v>-45.9</v>
       </c>
       <c r="F4" t="n">
-        <v>46</v>
+        <v>21.7</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>Declining</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SQL</t>
+          <t>JavaScript</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>7213</v>
+        <v>21005</v>
       </c>
       <c r="C5" t="n">
-        <v>5094</v>
+        <v>10581</v>
       </c>
       <c r="D5" t="n">
-        <v>-2119</v>
+        <v>-10424</v>
       </c>
       <c r="E5" t="n">
-        <v>-29.4</v>
+        <v>-49.6</v>
       </c>
       <c r="F5" t="n">
-        <v>44.1</v>
+        <v>21.5</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -1057,73 +1057,73 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3269</v>
+        <v>13859</v>
       </c>
       <c r="C6" t="n">
-        <v>4140</v>
+        <v>10099</v>
       </c>
       <c r="D6" t="n">
-        <v>871</v>
+        <v>-3760</v>
       </c>
       <c r="E6" t="n">
-        <v>26.6</v>
+        <v>-27.1</v>
       </c>
       <c r="F6" t="n">
-        <v>35.8</v>
+        <v>20.5</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Emerging</t>
+          <t>Declining</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C#</t>
+          <t>Rust</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4346</v>
+        <v>4724</v>
       </c>
       <c r="C7" t="n">
-        <v>3639</v>
+        <v>9262</v>
       </c>
       <c r="D7" t="n">
-        <v>-707</v>
+        <v>4538</v>
       </c>
       <c r="E7" t="n">
-        <v>-16.3</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="F7" t="n">
-        <v>31.5</v>
+        <v>18.8</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>Emerging</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Bash/Shell/PowerShell</t>
+          <t>Bash/Shell (all shells)</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4694</v>
+        <v>15503</v>
       </c>
       <c r="C8" t="n">
-        <v>3135</v>
+        <v>8662</v>
       </c>
       <c r="D8" t="n">
-        <v>-1559</v>
+        <v>-6841</v>
       </c>
       <c r="E8" t="n">
-        <v>-33.2</v>
+        <v>-44.1</v>
       </c>
       <c r="F8" t="n">
-        <v>27.1</v>
+        <v>17.6</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1134,216 +1134,945 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Go</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4556</v>
+        <v>5219</v>
       </c>
       <c r="C9" t="n">
-        <v>2987</v>
+        <v>7414</v>
       </c>
       <c r="D9" t="n">
-        <v>-1569</v>
+        <v>2195</v>
       </c>
       <c r="E9" t="n">
-        <v>-34.4</v>
+        <v>42.1</v>
       </c>
       <c r="F9" t="n">
-        <v>25.9</v>
+        <v>15.1</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Declining</t>
+          <t>Emerging</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Go</t>
+          <t>C#</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1133</v>
+        <v>8852</v>
       </c>
       <c r="C10" t="n">
-        <v>2813</v>
+        <v>6117</v>
       </c>
       <c r="D10" t="n">
-        <v>1680</v>
+        <v>-2735</v>
       </c>
       <c r="E10" t="n">
-        <v>148.3</v>
+        <v>-30.9</v>
       </c>
       <c r="F10" t="n">
-        <v>24.4</v>
+        <v>12.4</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Emerging</t>
+          <t>Declining</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Kotlin</t>
+          <t>C++</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>754</v>
+        <v>7485</v>
       </c>
       <c r="C11" t="n">
-        <v>1907</v>
+        <v>5243</v>
       </c>
       <c r="D11" t="n">
-        <v>1153</v>
+        <v>-2242</v>
       </c>
       <c r="E11" t="n">
-        <v>152.9</v>
+        <v>-30</v>
       </c>
       <c r="F11" t="n">
-        <v>16.5</v>
+        <v>10.7</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Emerging</t>
+          <t>Declining</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C++</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1964</v>
+        <v>9358</v>
       </c>
       <c r="C12" t="n">
-        <v>1645</v>
+        <v>4981</v>
       </c>
       <c r="D12" t="n">
-        <v>-319</v>
+        <v>-4377</v>
       </c>
       <c r="E12" t="n">
-        <v>-16.2</v>
+        <v>-46.8</v>
       </c>
       <c r="F12" t="n">
-        <v>14.2</v>
+        <v>10.1</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>Declining</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Rust</t>
+          <t>C</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>328</v>
+        <v>6987</v>
       </c>
       <c r="C13" t="n">
-        <v>1540</v>
+        <v>4548</v>
       </c>
       <c r="D13" t="n">
-        <v>1212</v>
+        <v>-2439</v>
       </c>
       <c r="E13" t="n">
-        <v>369.5</v>
+        <v>-34.9</v>
       </c>
       <c r="F13" t="n">
-        <v>13.3</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Emerging</t>
+          <t>Declining</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PHP</t>
+          <t>Kotlin</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>2950</v>
+        <v>3420</v>
       </c>
       <c r="C14" t="n">
-        <v>1475</v>
+        <v>3786</v>
       </c>
       <c r="D14" t="n">
-        <v>-1475</v>
+        <v>366</v>
       </c>
       <c r="E14" t="n">
-        <v>-50</v>
+        <v>10.7</v>
       </c>
       <c r="F14" t="n">
-        <v>12.8</v>
+        <v>7.7</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Declining</t>
+          <t>Stable</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>WebAssembly</t>
+          <t>PowerShell</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>136</v>
+        <v>7371</v>
       </c>
       <c r="C15" t="n">
-        <v>1417</v>
+        <v>3014</v>
       </c>
       <c r="D15" t="n">
-        <v>1281</v>
+        <v>-4357</v>
       </c>
       <c r="E15" t="n">
-        <v>941.9</v>
+        <v>-59.1</v>
       </c>
       <c r="F15" t="n">
-        <v>12.3</v>
+        <v>6.1</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Emerging</t>
+          <t>Declining</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>PHP</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1601</v>
+        <v>5994</v>
       </c>
       <c r="C16" t="n">
-        <v>1040</v>
+        <v>2873</v>
       </c>
       <c r="D16" t="n">
-        <v>-561</v>
+        <v>-3121</v>
       </c>
       <c r="E16" t="n">
-        <v>-35</v>
+        <v>-52.1</v>
       </c>
       <c r="F16" t="n">
-        <v>9</v>
+        <v>5.8</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
           <t>Declining</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Zig</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>680</v>
+      </c>
+      <c r="C17" t="n">
+        <v>2415</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1735</v>
+      </c>
+      <c r="E17" t="n">
+        <v>255.1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Emerging</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Lua</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>2910</v>
+      </c>
+      <c r="C18" t="n">
+        <v>2389</v>
+      </c>
+      <c r="D18" t="n">
+        <v>-521</v>
+      </c>
+      <c r="E18" t="n">
+        <v>-17.9</v>
+      </c>
+      <c r="F18" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Stable</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Assembly</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>2246</v>
+      </c>
+      <c r="C19" t="n">
+        <v>2154</v>
+      </c>
+      <c r="D19" t="n">
+        <v>-92</v>
+      </c>
+      <c r="E19" t="n">
+        <v>-4.1</v>
+      </c>
+      <c r="F19" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Stable</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Swift</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1719</v>
+      </c>
+      <c r="C20" t="n">
+        <v>2033</v>
+      </c>
+      <c r="D20" t="n">
+        <v>314</v>
+      </c>
+      <c r="E20" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="F20" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Stable</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Elixir</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>847</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1818</v>
+      </c>
+      <c r="D21" t="n">
+        <v>971</v>
+      </c>
+      <c r="E21" t="n">
+        <v>114.6</v>
+      </c>
+      <c r="F21" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Emerging</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Dart</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1885</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1653</v>
+      </c>
+      <c r="D22" t="n">
+        <v>-232</v>
+      </c>
+      <c r="E22" t="n">
+        <v>-12.3</v>
+      </c>
+      <c r="F22" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Stable</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Ruby</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>2046</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1587</v>
+      </c>
+      <c r="D23" t="n">
+        <v>-459</v>
+      </c>
+      <c r="E23" t="n">
+        <v>-22.4</v>
+      </c>
+      <c r="F23" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Declining</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1569</v>
+      </c>
+      <c r="C24" t="n">
+        <v>1308</v>
+      </c>
+      <c r="D24" t="n">
+        <v>-261</v>
+      </c>
+      <c r="E24" t="n">
+        <v>-16.6</v>
+      </c>
+      <c r="F24" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Stable</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Lisp</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>753</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1136</v>
+      </c>
+      <c r="D25" t="n">
+        <v>383</v>
+      </c>
+      <c r="E25" t="n">
+        <v>50.9</v>
+      </c>
+      <c r="F25" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Emerging</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>GDScript</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1062</v>
+      </c>
+      <c r="C26" t="n">
+        <v>1072</v>
+      </c>
+      <c r="D26" t="n">
+        <v>10</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F26" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Stable</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Gleam</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>354</v>
+      </c>
+      <c r="C27" t="n">
+        <v>972</v>
+      </c>
+      <c r="D27" t="n">
+        <v>618</v>
+      </c>
+      <c r="E27" t="n">
+        <v>174.6</v>
+      </c>
+      <c r="F27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Emerging</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Erlang</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>465</v>
+      </c>
+      <c r="C28" t="n">
+        <v>956</v>
+      </c>
+      <c r="D28" t="n">
+        <v>491</v>
+      </c>
+      <c r="E28" t="n">
+        <v>105.6</v>
+      </c>
+      <c r="F28" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Emerging</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Scala</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>843</v>
+      </c>
+      <c r="C29" t="n">
+        <v>924</v>
+      </c>
+      <c r="D29" t="n">
+        <v>81</v>
+      </c>
+      <c r="E29" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Stable</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>F#</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>406</v>
+      </c>
+      <c r="C30" t="n">
+        <v>908</v>
+      </c>
+      <c r="D30" t="n">
+        <v>502</v>
+      </c>
+      <c r="E30" t="n">
+        <v>123.6</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Emerging</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>OCaml</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>367</v>
+      </c>
+      <c r="C31" t="n">
+        <v>864</v>
+      </c>
+      <c r="D31" t="n">
+        <v>497</v>
+      </c>
+      <c r="E31" t="n">
+        <v>135.4</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Emerging</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>MicroPython</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>723</v>
+      </c>
+      <c r="C32" t="n">
+        <v>831</v>
+      </c>
+      <c r="D32" t="n">
+        <v>108</v>
+      </c>
+      <c r="E32" t="n">
+        <v>14.9</v>
+      </c>
+      <c r="F32" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Stable</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Perl</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1215</v>
+      </c>
+      <c r="C33" t="n">
+        <v>701</v>
+      </c>
+      <c r="D33" t="n">
+        <v>-514</v>
+      </c>
+      <c r="E33" t="n">
+        <v>-42.3</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Declining</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>MATLAB</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1231</v>
+      </c>
+      <c r="C34" t="n">
+        <v>617</v>
+      </c>
+      <c r="D34" t="n">
+        <v>-614</v>
+      </c>
+      <c r="E34" t="n">
+        <v>-49.9</v>
+      </c>
+      <c r="F34" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Declining</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Groovy</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1535</v>
+      </c>
+      <c r="C35" t="n">
+        <v>606</v>
+      </c>
+      <c r="D35" t="n">
+        <v>-929</v>
+      </c>
+      <c r="E35" t="n">
+        <v>-60.5</v>
+      </c>
+      <c r="F35" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Declining</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Visual Basic (.Net)</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1409</v>
+      </c>
+      <c r="C36" t="n">
+        <v>577</v>
+      </c>
+      <c r="D36" t="n">
+        <v>-832</v>
+      </c>
+      <c r="E36" t="n">
+        <v>-59</v>
+      </c>
+      <c r="F36" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Declining</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Mojo</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>145</v>
+      </c>
+      <c r="C37" t="n">
+        <v>572</v>
+      </c>
+      <c r="D37" t="n">
+        <v>427</v>
+      </c>
+      <c r="E37" t="n">
+        <v>294.5</v>
+      </c>
+      <c r="F37" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Emerging</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Delphi</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>796</v>
+      </c>
+      <c r="C38" t="n">
+        <v>563</v>
+      </c>
+      <c r="D38" t="n">
+        <v>-233</v>
+      </c>
+      <c r="E38" t="n">
+        <v>-29.3</v>
+      </c>
+      <c r="F38" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Declining</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Ada</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>431</v>
+      </c>
+      <c r="C39" t="n">
+        <v>511</v>
+      </c>
+      <c r="D39" t="n">
+        <v>80</v>
+      </c>
+      <c r="E39" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="F39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Stable</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>VBA</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1334</v>
+      </c>
+      <c r="C40" t="n">
+        <v>481</v>
+      </c>
+      <c r="D40" t="n">
+        <v>-853</v>
+      </c>
+      <c r="E40" t="n">
+        <v>-63.9</v>
+      </c>
+      <c r="F40" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Declining</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Prolog</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>338</v>
+      </c>
+      <c r="C41" t="n">
+        <v>414</v>
+      </c>
+      <c r="D41" t="n">
+        <v>76</v>
+      </c>
+      <c r="E41" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Emerging</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>COBOL</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>308</v>
+      </c>
+      <c r="C42" t="n">
+        <v>403</v>
+      </c>
+      <c r="D42" t="n">
+        <v>95</v>
+      </c>
+      <c r="E42" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Emerging</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Fortran</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>449</v>
+      </c>
+      <c r="C43" t="n">
+        <v>397</v>
+      </c>
+      <c r="D43" t="n">
+        <v>-52</v>
+      </c>
+      <c r="E43" t="n">
+        <v>-11.6</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Stable</t>
         </is>
       </c>
     </row>
@@ -1358,7 +2087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1405,19 +2134,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4153</v>
+        <v>14529</v>
       </c>
       <c r="C2" t="n">
-        <v>4386</v>
+        <v>11863</v>
       </c>
       <c r="D2" t="n">
-        <v>233</v>
+        <v>-2666</v>
       </c>
       <c r="E2" t="n">
-        <v>5.6</v>
+        <v>-18.3</v>
       </c>
       <c r="F2" t="n">
-        <v>38</v>
+        <v>24.1</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -1428,27 +2157,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MongoDB</t>
+          <t>SQLite</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3058</v>
+        <v>9798</v>
       </c>
       <c r="C3" t="n">
-        <v>3703</v>
+        <v>7185</v>
       </c>
       <c r="D3" t="n">
-        <v>645</v>
+        <v>-2613</v>
       </c>
       <c r="E3" t="n">
-        <v>21.1</v>
+        <v>-26.7</v>
       </c>
       <c r="F3" t="n">
-        <v>32.1</v>
+        <v>14.6</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Emerging</t>
+          <t>Declining</t>
         </is>
       </c>
     </row>
@@ -1459,23 +2188,23 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2536</v>
+        <v>7316</v>
       </c>
       <c r="C4" t="n">
-        <v>3385</v>
+        <v>6014</v>
       </c>
       <c r="D4" t="n">
-        <v>849</v>
+        <v>-1302</v>
       </c>
       <c r="E4" t="n">
-        <v>33.5</v>
+        <v>-17.8</v>
       </c>
       <c r="F4" t="n">
-        <v>29.3</v>
+        <v>12.2</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Emerging</t>
+          <t>Stable</t>
         </is>
       </c>
     </row>
@@ -1486,19 +2215,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5549</v>
+        <v>10581</v>
       </c>
       <c r="C5" t="n">
-        <v>3328</v>
+        <v>5120</v>
       </c>
       <c r="D5" t="n">
-        <v>-2221</v>
+        <v>-5461</v>
       </c>
       <c r="E5" t="n">
-        <v>-40</v>
+        <v>-51.6</v>
       </c>
       <c r="F5" t="n">
-        <v>28.8</v>
+        <v>10.4</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -1509,27 +2238,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Elasticsearch</t>
+          <t>MongoDB</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1980</v>
+        <v>6267</v>
       </c>
       <c r="C6" t="n">
-        <v>2898</v>
+        <v>4421</v>
       </c>
       <c r="D6" t="n">
-        <v>918</v>
+        <v>-1846</v>
       </c>
       <c r="E6" t="n">
-        <v>46.4</v>
+        <v>-29.5</v>
       </c>
       <c r="F6" t="n">
-        <v>25.1</v>
+        <v>9</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Emerging</t>
+          <t>Declining</t>
         </is>
       </c>
     </row>
@@ -1540,19 +2269,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4170</v>
+        <v>7871</v>
       </c>
       <c r="C7" t="n">
-        <v>2747</v>
+        <v>3851</v>
       </c>
       <c r="D7" t="n">
-        <v>-1423</v>
+        <v>-4020</v>
       </c>
       <c r="E7" t="n">
-        <v>-34.1</v>
+        <v>-51.1</v>
       </c>
       <c r="F7" t="n">
-        <v>23.8</v>
+        <v>7.8</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1563,23 +2292,23 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SQLite</t>
+          <t>Elasticsearch</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3292</v>
+        <v>4347</v>
       </c>
       <c r="C8" t="n">
-        <v>2465</v>
+        <v>3288</v>
       </c>
       <c r="D8" t="n">
-        <v>-827</v>
+        <v>-1059</v>
       </c>
       <c r="E8" t="n">
-        <v>-25.1</v>
+        <v>-24.4</v>
       </c>
       <c r="F8" t="n">
-        <v>21.3</v>
+        <v>6.7</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1590,104 +2319,104 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Firebase</t>
+          <t>MariaDB</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1343</v>
+        <v>5862</v>
       </c>
       <c r="C9" t="n">
-        <v>1679</v>
+        <v>3239</v>
       </c>
       <c r="D9" t="n">
-        <v>336</v>
+        <v>-2623</v>
       </c>
       <c r="E9" t="n">
-        <v>25</v>
+        <v>-44.7</v>
       </c>
       <c r="F9" t="n">
-        <v>14.5</v>
+        <v>6.6</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Emerging</t>
+          <t>Declining</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MariaDB</t>
+          <t>Dynamodb</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1724</v>
+        <v>2551</v>
       </c>
       <c r="C10" t="n">
-        <v>1400</v>
+        <v>1741</v>
       </c>
       <c r="D10" t="n">
-        <v>-324</v>
+        <v>-810</v>
       </c>
       <c r="E10" t="n">
-        <v>-18.8</v>
+        <v>-31.8</v>
       </c>
       <c r="F10" t="n">
-        <v>12.1</v>
+        <v>3.5</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>Declining</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>DynamoDB</t>
+          <t>Supabase</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>839</v>
+        <v>1558</v>
       </c>
       <c r="C11" t="n">
-        <v>1056</v>
+        <v>1621</v>
       </c>
       <c r="D11" t="n">
-        <v>217</v>
+        <v>63</v>
       </c>
       <c r="E11" t="n">
-        <v>25.9</v>
+        <v>4</v>
       </c>
       <c r="F11" t="n">
-        <v>9.1</v>
+        <v>3.3</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Emerging</t>
+          <t>Stable</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Cassandra</t>
+          <t>DuckDB</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>403</v>
+        <v>863</v>
       </c>
       <c r="C12" t="n">
-        <v>1023</v>
+        <v>1436</v>
       </c>
       <c r="D12" t="n">
-        <v>620</v>
+        <v>573</v>
       </c>
       <c r="E12" t="n">
-        <v>153.8</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="F12" t="n">
-        <v>8.9</v>
+        <v>2.9</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1698,27 +2427,513 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>BigQuery</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1705</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1371</v>
+      </c>
+      <c r="D13" t="n">
+        <v>-334</v>
+      </c>
+      <c r="E13" t="n">
+        <v>-19.6</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Stable</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>Oracle</t>
         </is>
       </c>
-      <c r="B13" t="n">
-        <v>1761</v>
-      </c>
-      <c r="C13" t="n">
-        <v>881</v>
-      </c>
-      <c r="D13" t="n">
-        <v>-880</v>
-      </c>
-      <c r="E13" t="n">
-        <v>-50</v>
-      </c>
-      <c r="F13" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="G13" t="inlineStr">
+      <c r="B14" t="n">
+        <v>2761</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1259</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-1502</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-54.4</v>
+      </c>
+      <c r="F14" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="G14" t="inlineStr">
         <is>
           <t>Declining</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Valkey</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>632</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1240</v>
+      </c>
+      <c r="D15" t="n">
+        <v>608</v>
+      </c>
+      <c r="E15" t="n">
+        <v>96.2</v>
+      </c>
+      <c r="F15" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Emerging</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Cassandra</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>766</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1214</v>
+      </c>
+      <c r="D16" t="n">
+        <v>448</v>
+      </c>
+      <c r="E16" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="F16" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Emerging</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Snowflake</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1079</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1068</v>
+      </c>
+      <c r="D17" t="n">
+        <v>-11</v>
+      </c>
+      <c r="E17" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Stable</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Firebase Realtime Database</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1299</v>
+      </c>
+      <c r="C18" t="n">
+        <v>1010</v>
+      </c>
+      <c r="D18" t="n">
+        <v>-289</v>
+      </c>
+      <c r="E18" t="n">
+        <v>-22.2</v>
+      </c>
+      <c r="F18" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Declining</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Cosmos DB</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1190</v>
+      </c>
+      <c r="C19" t="n">
+        <v>988</v>
+      </c>
+      <c r="D19" t="n">
+        <v>-202</v>
+      </c>
+      <c r="E19" t="n">
+        <v>-17</v>
+      </c>
+      <c r="F19" t="n">
+        <v>2</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Stable</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Cloud Firestore</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1494</v>
+      </c>
+      <c r="C20" t="n">
+        <v>980</v>
+      </c>
+      <c r="D20" t="n">
+        <v>-514</v>
+      </c>
+      <c r="E20" t="n">
+        <v>-34.4</v>
+      </c>
+      <c r="F20" t="n">
+        <v>2</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Declining</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Neo4J</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>691</v>
+      </c>
+      <c r="C21" t="n">
+        <v>972</v>
+      </c>
+      <c r="D21" t="n">
+        <v>281</v>
+      </c>
+      <c r="E21" t="n">
+        <v>40.7</v>
+      </c>
+      <c r="F21" t="n">
+        <v>2</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Emerging</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Databricks SQL</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>895</v>
+      </c>
+      <c r="C22" t="n">
+        <v>874</v>
+      </c>
+      <c r="D22" t="n">
+        <v>-21</v>
+      </c>
+      <c r="E22" t="n">
+        <v>-2.3</v>
+      </c>
+      <c r="F22" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Stable</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Clickhouse</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>627</v>
+      </c>
+      <c r="C23" t="n">
+        <v>844</v>
+      </c>
+      <c r="D23" t="n">
+        <v>217</v>
+      </c>
+      <c r="E23" t="n">
+        <v>34.6</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Emerging</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>InfluxDB</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>963</v>
+      </c>
+      <c r="C24" t="n">
+        <v>721</v>
+      </c>
+      <c r="D24" t="n">
+        <v>-242</v>
+      </c>
+      <c r="E24" t="n">
+        <v>-25.1</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Declining</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Amazon Redshift</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>611</v>
+      </c>
+      <c r="C25" t="n">
+        <v>685</v>
+      </c>
+      <c r="D25" t="n">
+        <v>74</v>
+      </c>
+      <c r="E25" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Stable</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Cockroachdb</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>262</v>
+      </c>
+      <c r="C26" t="n">
+        <v>632</v>
+      </c>
+      <c r="D26" t="n">
+        <v>370</v>
+      </c>
+      <c r="E26" t="n">
+        <v>141.2</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Emerging</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>H2</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1303</v>
+      </c>
+      <c r="C27" t="n">
+        <v>620</v>
+      </c>
+      <c r="D27" t="n">
+        <v>-683</v>
+      </c>
+      <c r="E27" t="n">
+        <v>-52.4</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Declining</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Pocketbase</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>262</v>
+      </c>
+      <c r="C28" t="n">
+        <v>407</v>
+      </c>
+      <c r="D28" t="n">
+        <v>145</v>
+      </c>
+      <c r="E28" t="n">
+        <v>55.3</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Emerging</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Microsoft Access</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>1244</v>
+      </c>
+      <c r="C29" t="n">
+        <v>363</v>
+      </c>
+      <c r="D29" t="n">
+        <v>-881</v>
+      </c>
+      <c r="E29" t="n">
+        <v>-70.8</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Declining</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>IBM DB2</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>615</v>
+      </c>
+      <c r="C30" t="n">
+        <v>330</v>
+      </c>
+      <c r="D30" t="n">
+        <v>-285</v>
+      </c>
+      <c r="E30" t="n">
+        <v>-46.3</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Declining</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Datomic</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>148</v>
+      </c>
+      <c r="C31" t="n">
+        <v>272</v>
+      </c>
+      <c r="D31" t="n">
+        <v>124</v>
+      </c>
+      <c r="E31" t="n">
+        <v>83.8</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Emerging</t>
         </is>
       </c>
     </row>
@@ -2200,7 +3415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2233,324 +3448,780 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Clojure</t>
+          <t>Ruby</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>152</v>
+        <v>1550</v>
       </c>
       <c r="C2" t="n">
-        <v>93404</v>
+        <v>102961</v>
       </c>
       <c r="D2" t="n">
-        <v>114203</v>
+        <v>114831</v>
       </c>
       <c r="E2" t="n">
-        <v>44.1</v>
+        <v>29.5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Go</t>
+          <t>Erlang</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1060</v>
+        <v>314</v>
       </c>
       <c r="C3" t="n">
-        <v>80000</v>
+        <v>100000</v>
       </c>
       <c r="D3" t="n">
-        <v>98923</v>
+        <v>108905</v>
       </c>
       <c r="E3" t="n">
-        <v>24.8</v>
+        <v>22.8</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Scala</t>
+          <t>Perl</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>461</v>
+        <v>806</v>
       </c>
       <c r="C4" t="n">
-        <v>79163</v>
+        <v>99886</v>
       </c>
       <c r="D4" t="n">
-        <v>98884</v>
+        <v>112073</v>
       </c>
       <c r="E4" t="n">
-        <v>24.7</v>
+        <v>26.4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ruby</t>
+          <t>Elixir</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1094</v>
+        <v>615</v>
       </c>
       <c r="C5" t="n">
-        <v>75000</v>
+        <v>99194</v>
       </c>
       <c r="D5" t="n">
-        <v>94376</v>
+        <v>109543</v>
       </c>
       <c r="E5" t="n">
-        <v>19</v>
+        <v>23.5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Elixir</t>
+          <t>Scala</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>169</v>
+        <v>600</v>
       </c>
       <c r="C6" t="n">
-        <v>71966</v>
+        <v>96524</v>
       </c>
       <c r="D6" t="n">
-        <v>89015</v>
+        <v>114361</v>
       </c>
       <c r="E6" t="n">
-        <v>12.3</v>
+        <v>28.9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Rust</t>
+          <t>Swift</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>311</v>
+        <v>1198</v>
       </c>
       <c r="C7" t="n">
-        <v>70000</v>
+        <v>92000</v>
       </c>
       <c r="D7" t="n">
-        <v>88382</v>
+        <v>104009</v>
       </c>
       <c r="E7" t="n">
-        <v>11.5</v>
+        <v>17.3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Bash/Shell/PowerShell</t>
+          <t>Groovy</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4417</v>
+        <v>1171</v>
       </c>
       <c r="C8" t="n">
-        <v>68745</v>
+        <v>90233</v>
       </c>
       <c r="D8" t="n">
-        <v>89946</v>
+        <v>101916</v>
       </c>
       <c r="E8" t="n">
-        <v>13.5</v>
+        <v>14.9</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Objective-C</t>
+          <t>Lisp</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>483</v>
+        <v>459</v>
       </c>
       <c r="C9" t="n">
-        <v>64115</v>
+        <v>90000</v>
       </c>
       <c r="D9" t="n">
-        <v>87429</v>
+        <v>107780</v>
       </c>
       <c r="E9" t="n">
-        <v>10.3</v>
+        <v>21.5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>Go</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4293</v>
+        <v>3783</v>
       </c>
       <c r="C10" t="n">
-        <v>64000</v>
+        <v>89815</v>
       </c>
       <c r="D10" t="n">
-        <v>85750</v>
+        <v>105716</v>
       </c>
       <c r="E10" t="n">
-        <v>8.199999999999999</v>
+        <v>19.2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>Bash/Shell (all shells)</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>552</v>
+        <v>11104</v>
       </c>
       <c r="C11" t="n">
-        <v>63016</v>
+        <v>83531</v>
       </c>
       <c r="D11" t="n">
-        <v>85477</v>
+        <v>97342</v>
       </c>
       <c r="E11" t="n">
-        <v>7.8</v>
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Swift</t>
+          <t>Rust</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>668</v>
+        <v>3117</v>
       </c>
       <c r="C12" t="n">
-        <v>60674</v>
+        <v>83000</v>
       </c>
       <c r="D12" t="n">
-        <v>81501</v>
+        <v>101345</v>
       </c>
       <c r="E12" t="n">
-        <v>2.8</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>Zig</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3012</v>
+        <v>399</v>
       </c>
       <c r="C13" t="n">
-        <v>60173</v>
+        <v>81210</v>
       </c>
       <c r="D13" t="n">
-        <v>80456</v>
+        <v>96562</v>
       </c>
       <c r="E13" t="n">
-        <v>3.5</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>C#</t>
+          <t>PowerShell</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3993</v>
+        <v>5334</v>
       </c>
       <c r="C14" t="n">
-        <v>59112</v>
+        <v>80992</v>
       </c>
       <c r="D14" t="n">
-        <v>79957</v>
+        <v>89809</v>
       </c>
       <c r="E14" t="n">
-        <v>1.6</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>JavaScript</t>
+          <t>Kotlin</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>8136</v>
+        <v>2428</v>
       </c>
       <c r="C15" t="n">
-        <v>58000</v>
+        <v>80152</v>
       </c>
       <c r="D15" t="n">
-        <v>79063</v>
+        <v>93572</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SQL</t>
+          <t>F#</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>6687</v>
+        <v>262</v>
       </c>
       <c r="C16" t="n">
-        <v>58284</v>
+        <v>80127</v>
       </c>
       <c r="D16" t="n">
-        <v>78852</v>
+        <v>91521</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.7</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>TypeScript</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>4168</v>
+        <v>10336</v>
       </c>
       <c r="C17" t="n">
-        <v>53437</v>
+        <v>79648</v>
       </c>
       <c r="D17" t="n">
-        <v>75838</v>
+        <v>92141</v>
       </c>
       <c r="E17" t="n">
-        <v>-7.6</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>C#</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>6397</v>
+      </c>
+      <c r="C18" t="n">
+        <v>78616</v>
+      </c>
+      <c r="D18" t="n">
+        <v>89654</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Gleam</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>209</v>
+      </c>
+      <c r="C19" t="n">
+        <v>77730</v>
+      </c>
+      <c r="D19" t="n">
+        <v>90917</v>
+      </c>
+      <c r="E19" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>12730</v>
+      </c>
+      <c r="C20" t="n">
+        <v>76828</v>
+      </c>
+      <c r="D20" t="n">
+        <v>92689</v>
+      </c>
+      <c r="E20" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SQL</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>13546</v>
+      </c>
+      <c r="C21" t="n">
+        <v>76518</v>
+      </c>
+      <c r="D21" t="n">
+        <v>90007</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>JavaScript</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>14873</v>
+      </c>
+      <c r="C22" t="n">
+        <v>75410</v>
+      </c>
+      <c r="D22" t="n">
+        <v>88540</v>
+      </c>
+      <c r="E22" t="n">
+        <v>-0.2</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>OCaml</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>199</v>
+      </c>
+      <c r="C23" t="n">
+        <v>75410</v>
+      </c>
+      <c r="D23" t="n">
+        <v>99022</v>
+      </c>
+      <c r="E23" t="n">
+        <v>11.6</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Lua</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1857</v>
+      </c>
+      <c r="C24" t="n">
+        <v>75320</v>
+      </c>
+      <c r="D24" t="n">
+        <v>92640</v>
+      </c>
+      <c r="E24" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Java</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>6283</v>
+      </c>
+      <c r="C25" t="n">
+        <v>75109</v>
+      </c>
+      <c r="D25" t="n">
+        <v>89963</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>C++</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>4605</v>
+      </c>
+      <c r="C26" t="n">
+        <v>74249</v>
+      </c>
+      <c r="D26" t="n">
+        <v>90234</v>
+      </c>
+      <c r="E26" t="n">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>HTML/CSS</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>13782</v>
+      </c>
+      <c r="C27" t="n">
+        <v>74000</v>
+      </c>
+      <c r="D27" t="n">
+        <v>86575</v>
+      </c>
+      <c r="E27" t="n">
+        <v>-2.4</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Fortran</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>271</v>
+      </c>
+      <c r="C28" t="n">
+        <v>73516</v>
+      </c>
+      <c r="D28" t="n">
+        <v>87466</v>
+      </c>
+      <c r="E28" t="n">
+        <v>-1.4</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>4095</v>
+      </c>
+      <c r="C29" t="n">
+        <v>72958</v>
+      </c>
+      <c r="D29" t="n">
+        <v>88707</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>VBA</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>908</v>
+      </c>
+      <c r="C30" t="n">
+        <v>71814</v>
+      </c>
+      <c r="D30" t="n">
+        <v>85025</v>
+      </c>
+      <c r="E30" t="n">
+        <v>-4.1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>MicroPython</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>408</v>
+      </c>
+      <c r="C31" t="n">
+        <v>70705</v>
+      </c>
+      <c r="D31" t="n">
+        <v>87409</v>
+      </c>
+      <c r="E31" t="n">
+        <v>-1.4</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1011</v>
+      </c>
+      <c r="C32" t="n">
+        <v>70000</v>
+      </c>
+      <c r="D32" t="n">
+        <v>86542</v>
+      </c>
+      <c r="E32" t="n">
+        <v>-2.4</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Assembly</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1187</v>
+      </c>
+      <c r="C33" t="n">
+        <v>69609</v>
+      </c>
+      <c r="D33" t="n">
+        <v>86517</v>
+      </c>
+      <c r="E33" t="n">
+        <v>-2.5</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>GDScript</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>622</v>
+      </c>
+      <c r="C34" t="n">
+        <v>68036</v>
+      </c>
+      <c r="D34" t="n">
+        <v>84956</v>
+      </c>
+      <c r="E34" t="n">
+        <v>-4.2</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Delphi</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>471</v>
+      </c>
+      <c r="C35" t="n">
+        <v>67655</v>
+      </c>
+      <c r="D35" t="n">
+        <v>73985</v>
+      </c>
+      <c r="E35" t="n">
+        <v>-16.6</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Visual Basic (.Net)</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>966</v>
+      </c>
+      <c r="C36" t="n">
+        <v>65462</v>
+      </c>
+      <c r="D36" t="n">
+        <v>74567</v>
+      </c>
+      <c r="E36" t="n">
+        <v>-15.9</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>PHP</t>
         </is>
       </c>
-      <c r="B18" t="n">
-        <v>2720</v>
-      </c>
-      <c r="C18" t="n">
-        <v>43296</v>
-      </c>
-      <c r="D18" t="n">
-        <v>66879</v>
-      </c>
-      <c r="E18" t="n">
-        <v>-25.2</v>
+      <c r="B37" t="n">
+        <v>4097</v>
+      </c>
+      <c r="C37" t="n">
+        <v>60000</v>
+      </c>
+      <c r="D37" t="n">
+        <v>72099</v>
+      </c>
+      <c r="E37" t="n">
+        <v>-18.7</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>MATLAB</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>700</v>
+      </c>
+      <c r="C38" t="n">
+        <v>58007</v>
+      </c>
+      <c r="D38" t="n">
+        <v>75035</v>
+      </c>
+      <c r="E38" t="n">
+        <v>-15.4</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>COBOL</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>182</v>
+      </c>
+      <c r="C39" t="n">
+        <v>58007</v>
+      </c>
+      <c r="D39" t="n">
+        <v>75772</v>
+      </c>
+      <c r="E39" t="n">
+        <v>-14.6</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Dart</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1201</v>
+      </c>
+      <c r="C40" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D40" t="n">
+        <v>70558</v>
+      </c>
+      <c r="E40" t="n">
+        <v>-20.4</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Prolog</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>172</v>
+      </c>
+      <c r="C41" t="n">
+        <v>49886</v>
+      </c>
+      <c r="D41" t="n">
+        <v>80150</v>
+      </c>
+      <c r="E41" t="n">
+        <v>-9.6</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Ada</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>216</v>
+      </c>
+      <c r="C42" t="n">
+        <v>44245</v>
+      </c>
+      <c r="D42" t="n">
+        <v>65346</v>
+      </c>
+      <c r="E42" t="n">
+        <v>-26.3</v>
       </c>
     </row>
   </sheetData>
@@ -2601,13 +4272,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6928</v>
+        <v>12351</v>
       </c>
       <c r="C2" t="n">
-        <v>59000</v>
+        <v>71078</v>
       </c>
       <c r="D2" t="n">
-        <v>72.90000000000001</v>
+        <v>77.2</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -2622,13 +4293,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6290</v>
+        <v>6453</v>
       </c>
       <c r="C3" t="n">
-        <v>56715</v>
+        <v>78616</v>
       </c>
       <c r="D3" t="n">
-        <v>65.90000000000001</v>
+        <v>46.1</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -2639,59 +4310,59 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DevOps Specialist</t>
+          <t>Product/BA</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1639</v>
+        <v>1273</v>
       </c>
       <c r="C4" t="n">
-        <v>71036</v>
+        <v>122171</v>
       </c>
       <c r="D4" t="n">
-        <v>46.1</v>
+        <v>35.4</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Priority 2</t>
+          <t>Priority 3</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Front-end Developer</t>
+          <t>DevOps Specialist</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3920</v>
+        <v>1053</v>
       </c>
       <c r="C5" t="n">
-        <v>53437</v>
+        <v>87011</v>
       </c>
       <c r="D5" t="n">
-        <v>45.2</v>
+        <v>18.4</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Priority 2</t>
+          <t>Priority 3</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Product/BA</t>
+          <t>Data Scientist / ML</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1179</v>
+        <v>574</v>
       </c>
       <c r="C6" t="n">
-        <v>61650</v>
+        <v>81210</v>
       </c>
       <c r="D6" t="n">
-        <v>33.3</v>
+        <v>13</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -2702,17 +4373,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Data/BI Analyst</t>
+          <t>Mobile Developer</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>802</v>
+        <v>1391</v>
       </c>
       <c r="C7" t="n">
-        <v>61872</v>
+        <v>69609</v>
       </c>
       <c r="D7" t="n">
-        <v>30.8</v>
+        <v>12.6</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -2723,17 +4394,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Data Scientist / ML</t>
+          <t>Front-end Developer</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>803</v>
+        <v>1974</v>
       </c>
       <c r="C8" t="n">
-        <v>60000</v>
+        <v>61362</v>
       </c>
       <c r="D8" t="n">
-        <v>28.9</v>
+        <v>12.3</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -2744,17 +4415,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Mobile Developer</t>
+          <t>Data/BI Analyst</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1959</v>
+        <v>351</v>
       </c>
       <c r="C9" t="n">
-        <v>46152</v>
+        <v>55000</v>
       </c>
       <c r="D9" t="n">
-        <v>23.5</v>
+        <v>0</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -2800,101 +4471,101 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3173</v>
+        <v>7233</v>
       </c>
       <c r="C2" t="n">
-        <v>27.5</v>
+        <v>14.7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>911</v>
+        <v>3025</v>
       </c>
       <c r="C3" t="n">
-        <v>7.9</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>India</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>841</v>
+        <v>2547</v>
       </c>
       <c r="C4" t="n">
-        <v>7.3</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>715</v>
+        <v>2042</v>
       </c>
       <c r="C5" t="n">
-        <v>6.2</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>France</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>442</v>
+        <v>1409</v>
       </c>
       <c r="C6" t="n">
-        <v>3.8</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>339</v>
+        <v>1305</v>
       </c>
       <c r="C7" t="n">
-        <v>2.9</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Ukraine</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>328</v>
+        <v>964</v>
       </c>
       <c r="C8" t="n">
-        <v>2.8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>287</v>
+        <v>888</v>
       </c>
       <c r="C9" t="n">
-        <v>2.5</v>
+        <v>1.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>